<commit_message>
feat: commit all pending changes — login redesign, dashboard, sidebar, BU Head, auth, leave requests, reports
- Redesigned login and reset password pages with Aress PMS branding
- Updated dashboard: new StatCard design, DashboardPage layout
- Updated Sidebar and AppLayout
- Auth: updated controller, service, JWT strategy, response DTO
- Dashboard backend: updated controller and service
- Leave requests: updated controller and service
- Frontend: updated auth API, client, WorkItemModal, BillingReportPage, useFeatureVisibility
- Added frontend public assets (pms-logo, login-img)
- Updated GitHub Actions deploy workflow
- Added F-056 BU Head role requirements, test cases, and test reports
- Updated consolidated test report
- Added KPI documentation and design system assets

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Document/KPI/Digital Appraisal System.xlsx
+++ b/Document/KPI/Digital Appraisal System.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\AI\Claude AI\Claude Code Advanced\project-management-system\Document\KPI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDAF079C-31FB-4AD8-97A3-B95B98646EF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48A8E60F-9E05-4C31-8E75-6BD828CEA8C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="KPI &amp; Scoring" sheetId="1" r:id="rId1"/>
@@ -1220,24 +1220,6 @@
     <xf numFmtId="0" fontId="4" fillId="8" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1280,9 +1262,6 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="8" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1294,9 +1273,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="8" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1310,14 +1286,8 @@
     <xf numFmtId="0" fontId="8" fillId="5" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1330,6 +1300,36 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1584,7 +1584,7 @@
       <c r="G1" s="7"/>
     </row>
     <row r="2" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="83" t="s">
+      <c r="A2" s="91" t="s">
         <v>60</v>
       </c>
       <c r="B2" s="8" t="s">
@@ -1606,7 +1606,7 @@
       <c r="G2" s="7"/>
     </row>
     <row r="3" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="66"/>
+      <c r="A3" s="92"/>
       <c r="B3" s="13" t="s">
         <v>7</v>
       </c>
@@ -1626,7 +1626,7 @@
       <c r="G3" s="7"/>
     </row>
     <row r="4" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="66"/>
+      <c r="A4" s="92"/>
       <c r="B4" s="13" t="s">
         <v>8</v>
       </c>
@@ -1646,7 +1646,7 @@
       <c r="G4" s="7"/>
     </row>
     <row r="5" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="67"/>
+      <c r="A5" s="93"/>
       <c r="B5" s="13" t="s">
         <v>9</v>
       </c>
@@ -1666,7 +1666,7 @@
       <c r="G5" s="7"/>
     </row>
     <row r="6" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="83" t="s">
+      <c r="A6" s="91" t="s">
         <v>61</v>
       </c>
       <c r="B6" s="8" t="s">
@@ -1688,7 +1688,7 @@
       <c r="G6" s="7"/>
     </row>
     <row r="7" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="66"/>
+      <c r="A7" s="92"/>
       <c r="B7" s="13" t="s">
         <v>55</v>
       </c>
@@ -1703,7 +1703,7 @@
       <c r="G7" s="7"/>
     </row>
     <row r="8" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="67"/>
+      <c r="A8" s="93"/>
       <c r="B8" s="13" t="s">
         <v>56</v>
       </c>
@@ -1718,10 +1718,10 @@
       <c r="G8" s="7"/>
     </row>
     <row r="9" spans="1:7" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A9" s="83" t="s">
+      <c r="A9" s="91" t="s">
         <v>62</v>
       </c>
-      <c r="B9" s="87" t="s">
+      <c r="B9" s="78" t="s">
         <v>50</v>
       </c>
       <c r="C9" s="9">
@@ -1735,7 +1735,7 @@
       <c r="G9" s="7"/>
     </row>
     <row r="10" spans="1:7" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="67"/>
+      <c r="A10" s="93"/>
       <c r="B10" s="22" t="s">
         <v>63</v>
       </c>
@@ -1750,10 +1750,10 @@
       <c r="G10" s="7"/>
     </row>
     <row r="11" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="83" t="s">
+      <c r="A11" s="91" t="s">
         <v>86</v>
       </c>
-      <c r="B11" s="86" t="s">
+      <c r="B11" s="77" t="s">
         <v>57</v>
       </c>
       <c r="C11" s="9">
@@ -1767,8 +1767,8 @@
       <c r="G11" s="7"/>
     </row>
     <row r="12" spans="1:7" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="67"/>
-      <c r="B12" s="92" t="s">
+      <c r="A12" s="93"/>
+      <c r="B12" s="82" t="s">
         <v>11</v>
       </c>
       <c r="C12" s="23">
@@ -1782,7 +1782,7 @@
       <c r="G12" s="7"/>
     </row>
     <row r="13" spans="1:7" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="94" t="s">
+      <c r="A13" s="75" t="s">
         <v>59</v>
       </c>
       <c r="B13" s="8" t="s">
@@ -1799,10 +1799,10 @@
       <c r="G13" s="7"/>
     </row>
     <row r="14" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="99" t="s">
+      <c r="A14" s="87" t="s">
         <v>67</v>
       </c>
-      <c r="B14" s="98" t="s">
+      <c r="B14" s="86" t="s">
         <v>13</v>
       </c>
       <c r="C14" s="9">
@@ -1816,10 +1816,10 @@
       <c r="G14" s="7"/>
     </row>
     <row r="15" spans="1:7" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="99" t="s">
+      <c r="A15" s="87" t="s">
         <v>66</v>
       </c>
-      <c r="B15" s="97"/>
+      <c r="B15" s="85"/>
       <c r="C15" s="23">
         <v>0.05</v>
       </c>
@@ -1831,10 +1831,10 @@
       <c r="G15" s="7"/>
     </row>
     <row r="16" spans="1:7" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="96" t="s">
+      <c r="A16" s="89" t="s">
         <v>14</v>
       </c>
-      <c r="B16" s="65"/>
+      <c r="B16" s="90"/>
       <c r="C16" s="25">
         <f>SUM(C2:C15)</f>
         <v>1.0000000000000002</v>
@@ -10763,20 +10763,20 @@
       <c r="D1" s="34" t="s">
         <v>25</v>
       </c>
-      <c r="E1" s="70" t="s">
+      <c r="E1" s="62" t="s">
         <v>26</v>
       </c>
-      <c r="F1" s="81" t="s">
+      <c r="F1" s="73" t="s">
         <v>84</v>
       </c>
-      <c r="G1" s="82" t="s">
+      <c r="G1" s="74" t="s">
         <v>85</v>
       </c>
-      <c r="H1" s="68"/>
-      <c r="I1" s="68"/>
+      <c r="H1" s="60"/>
+      <c r="I1" s="60"/>
     </row>
     <row r="2" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="60" t="s">
+      <c r="A2" s="94" t="s">
         <v>60</v>
       </c>
       <c r="B2" s="51" t="s">
@@ -10788,20 +10788,20 @@
       <c r="D2" s="53" t="s">
         <v>28</v>
       </c>
-      <c r="E2" s="71" t="s">
+      <c r="E2" s="63" t="s">
         <v>29</v>
       </c>
-      <c r="F2" s="74" t="s">
+      <c r="F2" s="66" t="s">
         <v>74</v>
       </c>
-      <c r="G2" s="79" t="s">
+      <c r="G2" s="71" t="s">
         <v>73</v>
       </c>
-      <c r="H2" s="68"/>
-      <c r="I2" s="68"/>
+      <c r="H2" s="60"/>
+      <c r="I2" s="60"/>
     </row>
     <row r="3" spans="1:9" ht="57.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="61"/>
+      <c r="A3" s="95"/>
       <c r="B3" s="54" t="s">
         <v>30</v>
       </c>
@@ -10811,20 +10811,20 @@
       <c r="D3" s="56" t="s">
         <v>31</v>
       </c>
-      <c r="E3" s="69" t="s">
+      <c r="E3" s="61" t="s">
         <v>32</v>
       </c>
-      <c r="F3" s="74" t="s">
+      <c r="F3" s="66" t="s">
         <v>70</v>
       </c>
-      <c r="G3" s="80" t="s">
+      <c r="G3" s="72" t="s">
         <v>71</v>
       </c>
-      <c r="H3" s="68"/>
-      <c r="I3" s="68"/>
+      <c r="H3" s="60"/>
+      <c r="I3" s="60"/>
     </row>
     <row r="4" spans="1:9" ht="97.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="61"/>
+      <c r="A4" s="95"/>
       <c r="B4" s="54" t="s">
         <v>33</v>
       </c>
@@ -10834,18 +10834,18 @@
       <c r="D4" s="56" t="s">
         <v>34</v>
       </c>
-      <c r="E4" s="69" t="s">
+      <c r="E4" s="61" t="s">
         <v>35</v>
       </c>
-      <c r="F4" s="74" t="s">
+      <c r="F4" s="66" t="s">
         <v>72</v>
       </c>
-      <c r="G4" s="79"/>
-      <c r="H4" s="68"/>
-      <c r="I4" s="68"/>
+      <c r="G4" s="71"/>
+      <c r="H4" s="60"/>
+      <c r="I4" s="60"/>
     </row>
     <row r="5" spans="1:9" ht="42.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="62"/>
+      <c r="A5" s="96"/>
       <c r="B5" s="57" t="s">
         <v>36</v>
       </c>
@@ -10855,20 +10855,20 @@
       <c r="D5" s="59" t="s">
         <v>37</v>
       </c>
-      <c r="E5" s="72" t="s">
+      <c r="E5" s="64" t="s">
         <v>38</v>
       </c>
-      <c r="F5" s="74" t="s">
+      <c r="F5" s="66" t="s">
         <v>69</v>
       </c>
-      <c r="G5" s="79" t="s">
+      <c r="G5" s="71" t="s">
         <v>73</v>
       </c>
-      <c r="H5" s="68"/>
-      <c r="I5" s="68"/>
+      <c r="H5" s="60"/>
+      <c r="I5" s="60"/>
     </row>
     <row r="6" spans="1:9" ht="86.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="60" t="s">
+      <c r="A6" s="94" t="s">
         <v>61</v>
       </c>
       <c r="B6" s="51" t="s">
@@ -10880,18 +10880,18 @@
       <c r="D6" s="53" t="s">
         <v>40</v>
       </c>
-      <c r="E6" s="71" t="s">
+      <c r="E6" s="63" t="s">
         <v>41</v>
       </c>
-      <c r="F6" s="74" t="s">
+      <c r="F6" s="66" t="s">
         <v>75</v>
       </c>
-      <c r="G6" s="79"/>
-      <c r="H6" s="68"/>
-      <c r="I6" s="68"/>
+      <c r="G6" s="71"/>
+      <c r="H6" s="60"/>
+      <c r="I6" s="60"/>
     </row>
     <row r="7" spans="1:9" ht="71.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="61"/>
+      <c r="A7" s="95"/>
       <c r="B7" s="56" t="s">
         <v>42</v>
       </c>
@@ -10901,18 +10901,18 @@
       <c r="D7" s="56" t="s">
         <v>43</v>
       </c>
-      <c r="E7" s="69" t="s">
+      <c r="E7" s="61" t="s">
         <v>81</v>
       </c>
-      <c r="F7" s="74" t="s">
+      <c r="F7" s="66" t="s">
         <v>82</v>
       </c>
-      <c r="G7" s="79"/>
-      <c r="H7" s="68"/>
-      <c r="I7" s="68"/>
+      <c r="G7" s="71"/>
+      <c r="H7" s="60"/>
+      <c r="I7" s="60"/>
     </row>
     <row r="8" spans="1:9" ht="79.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="61"/>
+      <c r="A8" s="95"/>
       <c r="B8" s="56" t="s">
         <v>44</v>
       </c>
@@ -10922,70 +10922,70 @@
       <c r="D8" s="56" t="s">
         <v>43</v>
       </c>
-      <c r="E8" s="69" t="s">
+      <c r="E8" s="61" t="s">
         <v>80</v>
       </c>
-      <c r="F8" s="74" t="s">
+      <c r="F8" s="66" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="79.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="84" t="s">
+      <c r="A9" s="97" t="s">
         <v>62</v>
       </c>
-      <c r="B9" s="88" t="s">
+      <c r="B9" s="79" t="s">
         <v>50</v>
       </c>
       <c r="C9" s="52">
         <v>0.05</v>
       </c>
-      <c r="D9" s="85" t="s">
+      <c r="D9" s="76" t="s">
         <v>51</v>
       </c>
-      <c r="E9" s="71" t="s">
+      <c r="E9" s="63" t="s">
         <v>52</v>
       </c>
-      <c r="F9" s="74" t="s">
+      <c r="F9" s="66" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="79.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="63"/>
-      <c r="B10" s="88" t="s">
+      <c r="A10" s="98"/>
+      <c r="B10" s="79" t="s">
         <v>63</v>
       </c>
       <c r="C10" s="52">
         <v>0.05</v>
       </c>
       <c r="D10" s="53"/>
-      <c r="E10" s="71" t="s">
+      <c r="E10" s="63" t="s">
         <v>64</v>
       </c>
-      <c r="F10" s="74" t="s">
+      <c r="F10" s="66" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="62.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="89" t="s">
+      <c r="A11" s="99" t="s">
         <v>68</v>
       </c>
-      <c r="B11" s="90" t="s">
+      <c r="B11" s="80" t="s">
         <v>57</v>
       </c>
       <c r="C11" s="47">
         <v>0.05</v>
       </c>
       <c r="D11" s="48"/>
-      <c r="E11" s="75" t="s">
+      <c r="E11" s="67" t="s">
         <v>58</v>
       </c>
-      <c r="F11" s="74" t="s">
+      <c r="F11" s="66" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="61.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="64"/>
-      <c r="B12" s="91" t="s">
+      <c r="A12" s="100"/>
+      <c r="B12" s="81" t="s">
         <v>11</v>
       </c>
       <c r="C12" s="49">
@@ -10994,10 +10994,10 @@
       <c r="D12" s="50" t="s">
         <v>45</v>
       </c>
-      <c r="E12" s="76" t="s">
+      <c r="E12" s="68" t="s">
         <v>46</v>
       </c>
-      <c r="F12" s="74" t="s">
+      <c r="F12" s="66" t="s">
         <v>78</v>
       </c>
     </row>
@@ -11005,7 +11005,7 @@
       <c r="A13" s="42" t="s">
         <v>59</v>
       </c>
-      <c r="B13" s="93" t="s">
+      <c r="B13" s="83" t="s">
         <v>47</v>
       </c>
       <c r="C13" s="43">
@@ -11014,15 +11014,15 @@
       <c r="D13" s="44" t="s">
         <v>48</v>
       </c>
-      <c r="E13" s="77" t="s">
+      <c r="E13" s="69" t="s">
         <v>49</v>
       </c>
-      <c r="F13" s="74" t="s">
+      <c r="F13" s="66" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="60.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="95" t="s">
+      <c r="A14" s="84" t="s">
         <v>67</v>
       </c>
       <c r="B14" s="39" t="s">
@@ -11034,15 +11034,15 @@
       <c r="D14" s="41" t="s">
         <v>54</v>
       </c>
-      <c r="E14" s="78" t="s">
+      <c r="E14" s="70" t="s">
         <v>65</v>
       </c>
-      <c r="F14" s="74" t="s">
+      <c r="F14" s="66" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="62.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="100" t="s">
+      <c r="A15" s="88" t="s">
         <v>66</v>
       </c>
       <c r="B15" s="45"/>
@@ -11050,8 +11050,8 @@
         <v>0.05</v>
       </c>
       <c r="D15" s="45"/>
-      <c r="E15" s="73"/>
-      <c r="F15" s="74" t="s">
+      <c r="E15" s="65"/>
+      <c r="F15" s="66" t="s">
         <v>78</v>
       </c>
     </row>

</xml_diff>